<commit_message>
Fixed for linux by using playwright instead of webdriver
</commit_message>
<xml_diff>
--- a/linkedin_leaderboards_Jul-2026.xlsx
+++ b/linkedin_leaderboards_Jul-2026.xlsx
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -51,7 +54,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,13 +62,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1286,7 +1295,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2:28</t>
+          <t>2:33</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1877,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2:36</t>
+          <t>2:42</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3030,11 @@
       <c r="R6" t="n">
         <v>3</v>
       </c>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3434,7 +3447,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>3:03</t>
+          <t>3:11</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4159,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1:49</t>
+          <t>1:53</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4465,11 @@
           <t>0:56</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1:10</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4825,7 +4842,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2:36</t>
+          <t>2:37</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5800,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1:41</t>
+          <t>1:46</t>
         </is>
       </c>
     </row>

</xml_diff>